<commit_message>
Sin coordenadas ni UBIGEO: las sedes se ubican por el nombre de su distrito
Se quitan LATITUD, LONGITUD y OBSERVACION de la hoja Organos; cada burbuja va al centro
de su distrito en el mapa.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018ZEyFKvQEhXemhLNvQ6ZCJ
</commit_message>
<xml_diff>
--- a/dashboard.xlsx
+++ b/dashboard.xlsx
@@ -173,9 +173,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="t_Organos" displayName="t_Organos" ref="A1:K102" headerRowCount="1">
-  <autoFilter ref="A1:K102"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="t_Organos" displayName="t_Organos" ref="A1:H102" headerRowCount="1">
+  <autoFilter ref="A1:H102"/>
+  <tableColumns count="8">
     <tableColumn id="1" name="CODIGO"/>
     <tableColumn id="2" name="DEPENDENCIA"/>
     <tableColumn id="3" name="ESPECIALIDAD"/>
@@ -184,9 +184,6 @@
     <tableColumn id="6" name="DEPARTAMENTO"/>
     <tableColumn id="7" name="PROVINCIA"/>
     <tableColumn id="8" name="DISTRITO"/>
-    <tableColumn id="9" name="LATITUD"/>
-    <tableColumn id="10" name="LONGITUD"/>
-    <tableColumn id="11" name="OBSERVACION"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showRowStripes="1"/>
 </table>
@@ -592,9 +589,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -630,9 +625,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
@@ -657,14 +650,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">                    SEDE_DISTRITO: el distrito donde está el juzgado (así sale la burbuja en el mapa).</t>
+          <t xml:space="preserve">                    SEDE_DISTRITO: el distrito donde está el juzgado (el mapa pone ahí la burbuja; no hacen falta coordenadas).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Organos           → tarjeta '101 órganos jurisdiccionales' y ubicación de las sedes (LATITUD / LONGITUD).</t>
+          <t>Organos           → tarjeta '101 órganos jurisdiccionales'. Un órgano por fila; DISTRITO es donde está la sede.</t>
         </is>
       </c>
     </row>
@@ -717,9 +710,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-    </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
@@ -737,7 +728,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>• Coordenadas con errores de tipeo corregidas en Organos (ver columna OBSERVACION): Chupaca, Concepción y El Tambo.</t>
+          <t>• Ya no se usan coordenadas ni UBIGEO: el mapa ubica cada sede por el nombre de su distrito.</t>
         </is>
       </c>
     </row>
@@ -9189,7 +9180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K102"/>
+  <dimension ref="A1:H102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -9246,21 +9237,6 @@
           <t>DISTRITO</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>LATITUD</t>
-        </is>
-      </c>
-      <c r="J1" s="3" t="inlineStr">
-        <is>
-          <t>LONGITUD</t>
-        </is>
-      </c>
-      <c r="K1" s="3" t="inlineStr">
-        <is>
-          <t>OBSERVACION</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9303,17 +9279,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I2" t="n">
-        <v>-12.059531</v>
-      </c>
-      <c r="J2" t="n">
-        <v>-75.21550000000001</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>longitud corregida (era -74.8881)</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9356,17 +9321,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I3" t="n">
-        <v>-12.059531</v>
-      </c>
-      <c r="J3" t="n">
-        <v>-75.21550000000001</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>longitud corregida (era -74.8881)</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9409,17 +9363,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I4" t="n">
-        <v>-12.059531</v>
-      </c>
-      <c r="J4" t="n">
-        <v>-75.21550000000001</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>longitud corregida (era -74.8881)</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9462,17 +9405,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I5" t="n">
-        <v>-12.059531</v>
-      </c>
-      <c r="J5" t="n">
-        <v>-75.21550000000001</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>longitud corregida (era -74.8881)</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9515,17 +9447,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I6" t="n">
-        <v>-12.059531</v>
-      </c>
-      <c r="J6" t="n">
-        <v>-75.21550000000001</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>longitud corregida (era -74.8881)</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -9568,17 +9489,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I7" t="n">
-        <v>-12.059531</v>
-      </c>
-      <c r="J7" t="n">
-        <v>-75.21550000000001</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>longitud corregida (era -74.8881)</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -9621,12 +9531,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I8" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J8" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -9669,12 +9573,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I9" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J9" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9717,12 +9615,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I10" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J10" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9765,12 +9657,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I11" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J11" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9813,12 +9699,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I12" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J12" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9861,12 +9741,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I13" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J13" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9909,12 +9783,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I14" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J14" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -9957,12 +9825,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I15" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J15" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -10005,12 +9867,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I16" t="n">
-        <v>-12.059261</v>
-      </c>
-      <c r="J16" t="n">
-        <v>-75.215339</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -10053,17 +9909,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I17" t="n">
-        <v>-12.059261</v>
-      </c>
-      <c r="J17" t="n">
-        <v>-75.215339</v>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>coordenada corregida (era -13.0593, -76.2153)</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -10106,12 +9951,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I18" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J18" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -10154,12 +9993,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I19" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J19" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -10202,12 +10035,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I20" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J20" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -10250,12 +10077,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I21" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J21" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -10298,12 +10119,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I22" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J22" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -10346,12 +10161,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I23" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J23" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -10394,12 +10203,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I24" t="n">
-        <v>-12.059261</v>
-      </c>
-      <c r="J24" t="n">
-        <v>-75.215339</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -10442,17 +10245,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I25" t="n">
-        <v>-12.059261</v>
-      </c>
-      <c r="J25" t="n">
-        <v>-75.215339</v>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>coordenada corregida (era -13.0593, -76.2153)</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -10495,17 +10287,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I26" t="n">
-        <v>-12.059261</v>
-      </c>
-      <c r="J26" t="n">
-        <v>-75.215339</v>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>coordenada corregida (era -14.0593, -77.2153)</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -10548,12 +10329,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I27" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J27" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -10596,12 +10371,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I28" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J28" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -10644,12 +10413,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I29" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J29" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -10692,12 +10455,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I30" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J30" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -10740,12 +10497,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I31" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J31" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -10788,12 +10539,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I32" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J32" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -10836,12 +10581,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I33" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J33" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -10884,12 +10623,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I34" t="n">
-        <v>-12.059261</v>
-      </c>
-      <c r="J34" t="n">
-        <v>-75.215339</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -10932,17 +10665,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I35" t="n">
-        <v>-12.059261</v>
-      </c>
-      <c r="J35" t="n">
-        <v>-75.215339</v>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>coordenada corregida (era -13.0593, -76.2153)</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -10985,17 +10707,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I36" t="n">
-        <v>-12.059261</v>
-      </c>
-      <c r="J36" t="n">
-        <v>-75.215339</v>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>coordenada corregida (era -14.0593, -77.2153)</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -11038,12 +10749,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I37" t="n">
-        <v>-12.060394</v>
-      </c>
-      <c r="J37" t="n">
-        <v>-75.215478</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -11086,12 +10791,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I38" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J38" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -11134,12 +10833,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I39" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J39" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -11182,12 +10875,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I40" t="n">
-        <v>-12.060394</v>
-      </c>
-      <c r="J40" t="n">
-        <v>-75.215478</v>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -11230,12 +10917,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I41" t="n">
-        <v>-12.060394</v>
-      </c>
-      <c r="J41" t="n">
-        <v>-75.215478</v>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -11278,12 +10959,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I42" t="n">
-        <v>-12.060381</v>
-      </c>
-      <c r="J42" t="n">
-        <v>-75.216983</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -11326,12 +11001,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I43" t="n">
-        <v>-12.060381</v>
-      </c>
-      <c r="J43" t="n">
-        <v>-75.216983</v>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -11374,12 +11043,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I44" t="n">
-        <v>-12.060381</v>
-      </c>
-      <c r="J44" t="n">
-        <v>-75.216983</v>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -11422,12 +11085,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I45" t="n">
-        <v>-12.060381</v>
-      </c>
-      <c r="J45" t="n">
-        <v>-75.216983</v>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -11470,12 +11127,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I46" t="n">
-        <v>-12.059022</v>
-      </c>
-      <c r="J46" t="n">
-        <v>-75.211078</v>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -11518,12 +11169,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I47" t="n">
-        <v>-12.059022</v>
-      </c>
-      <c r="J47" t="n">
-        <v>-75.211078</v>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -11566,12 +11211,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I48" t="n">
-        <v>-12.059022</v>
-      </c>
-      <c r="J48" t="n">
-        <v>-75.211078</v>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -11614,12 +11253,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I49" t="n">
-        <v>-12.059022</v>
-      </c>
-      <c r="J49" t="n">
-        <v>-75.211078</v>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -11662,12 +11295,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I50" t="n">
-        <v>-12.059022</v>
-      </c>
-      <c r="J50" t="n">
-        <v>-75.211078</v>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -11710,12 +11337,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I51" t="n">
-        <v>-12.059022</v>
-      </c>
-      <c r="J51" t="n">
-        <v>-75.211078</v>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -11758,12 +11379,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I52" t="n">
-        <v>-12.060397</v>
-      </c>
-      <c r="J52" t="n">
-        <v>-75.213447</v>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -11806,12 +11421,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I53" t="n">
-        <v>-12.060381</v>
-      </c>
-      <c r="J53" t="n">
-        <v>-75.216983</v>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -11854,12 +11463,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I54" t="n">
-        <v>-12.060381</v>
-      </c>
-      <c r="J54" t="n">
-        <v>-75.216983</v>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -11902,12 +11505,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I55" t="n">
-        <v>-12.059022</v>
-      </c>
-      <c r="J55" t="n">
-        <v>-75.211078</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -11950,12 +11547,6 @@
           <t>EL TAMBO</t>
         </is>
       </c>
-      <c r="I56" t="n">
-        <v>-12.059022</v>
-      </c>
-      <c r="J56" t="n">
-        <v>-75.211078</v>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -11998,12 +11589,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I57" t="n">
-        <v>-12.061481</v>
-      </c>
-      <c r="J57" t="n">
-        <v>-75.200372</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -12046,12 +11631,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I58" t="n">
-        <v>-12.060397</v>
-      </c>
-      <c r="J58" t="n">
-        <v>-75.213447</v>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -12094,12 +11673,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I59" t="n">
-        <v>-12.060397</v>
-      </c>
-      <c r="J59" t="n">
-        <v>-75.213447</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -12142,12 +11715,6 @@
           <t>HUANCAYO</t>
         </is>
       </c>
-      <c r="I60" t="n">
-        <v>-12.060397</v>
-      </c>
-      <c r="J60" t="n">
-        <v>-75.213447</v>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -12190,12 +11757,6 @@
           <t>CHILCA</t>
         </is>
       </c>
-      <c r="I61" t="n">
-        <v>-12.080644</v>
-      </c>
-      <c r="J61" t="n">
-        <v>-75.207767</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -12238,12 +11799,6 @@
           <t>CHILCA</t>
         </is>
       </c>
-      <c r="I62" t="n">
-        <v>-12.080644</v>
-      </c>
-      <c r="J62" t="n">
-        <v>-75.207767</v>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -12286,12 +11841,6 @@
           <t>SAN AGUSTIN</t>
         </is>
       </c>
-      <c r="I63" t="n">
-        <v>-11.986544</v>
-      </c>
-      <c r="J63" t="n">
-        <v>-75.242814</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -12334,17 +11883,6 @@
           <t>CHUPACA</t>
         </is>
       </c>
-      <c r="I64" t="n">
-        <v>-12.062139</v>
-      </c>
-      <c r="J64" t="n">
-        <v>-75.17975</v>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>longitud corregida (era -7517.975)</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -12387,17 +11925,6 @@
           <t>CHUPACA</t>
         </is>
       </c>
-      <c r="I65" t="n">
-        <v>-12.062139</v>
-      </c>
-      <c r="J65" t="n">
-        <v>-75.17975</v>
-      </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>longitud corregida (era -7517.975)</t>
-        </is>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -12440,17 +11967,6 @@
           <t>CHUPACA</t>
         </is>
       </c>
-      <c r="I66" t="n">
-        <v>-12.062139</v>
-      </c>
-      <c r="J66" t="n">
-        <v>-75.17975</v>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>longitud corregida (era -7517.975)</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -12493,17 +12009,6 @@
           <t>CHUPACA</t>
         </is>
       </c>
-      <c r="I67" t="n">
-        <v>-12.062139</v>
-      </c>
-      <c r="J67" t="n">
-        <v>-75.17975</v>
-      </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>longitud corregida (era -7517.975)</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -12546,17 +12051,6 @@
           <t>CHUPACA</t>
         </is>
       </c>
-      <c r="I68" t="n">
-        <v>-12.062139</v>
-      </c>
-      <c r="J68" t="n">
-        <v>-75.17975</v>
-      </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>longitud corregida (era -7517.975)</t>
-        </is>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -12599,12 +12093,6 @@
           <t>CONCEPCION</t>
         </is>
       </c>
-      <c r="I69" t="n">
-        <v>-11.926083</v>
-      </c>
-      <c r="J69" t="n">
-        <v>-75.310647</v>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -12647,17 +12135,6 @@
           <t>CONCEPCION</t>
         </is>
       </c>
-      <c r="I70" t="n">
-        <v>-11.926083</v>
-      </c>
-      <c r="J70" t="n">
-        <v>-75.310647</v>
-      </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>latitud corregida (era -12.9261)</t>
-        </is>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -12700,17 +12177,6 @@
           <t>CONCEPCION</t>
         </is>
       </c>
-      <c r="I71" t="n">
-        <v>-11.926083</v>
-      </c>
-      <c r="J71" t="n">
-        <v>-75.310647</v>
-      </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>latitud corregida (era -13.9261)</t>
-        </is>
-      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -12753,17 +12219,6 @@
           <t>CONCEPCION</t>
         </is>
       </c>
-      <c r="I72" t="n">
-        <v>-11.926083</v>
-      </c>
-      <c r="J72" t="n">
-        <v>-75.310647</v>
-      </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>latitud corregida (era -14.9261)</t>
-        </is>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -12806,12 +12261,6 @@
           <t>JAUJA</t>
         </is>
       </c>
-      <c r="I73" t="n">
-        <v>-11.7676</v>
-      </c>
-      <c r="J73" t="n">
-        <v>-75.497944</v>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -12854,12 +12303,6 @@
           <t>JAUJA</t>
         </is>
       </c>
-      <c r="I74" t="n">
-        <v>-11.7676</v>
-      </c>
-      <c r="J74" t="n">
-        <v>-75.497944</v>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -12902,12 +12345,6 @@
           <t>JAUJA</t>
         </is>
       </c>
-      <c r="I75" t="n">
-        <v>-11.7676</v>
-      </c>
-      <c r="J75" t="n">
-        <v>-75.497944</v>
-      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -12950,12 +12387,6 @@
           <t>JAUJA</t>
         </is>
       </c>
-      <c r="I76" t="n">
-        <v>-11.7676</v>
-      </c>
-      <c r="J76" t="n">
-        <v>-75.497944</v>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -12998,12 +12429,6 @@
           <t>JAUJA</t>
         </is>
       </c>
-      <c r="I77" t="n">
-        <v>-11.7676</v>
-      </c>
-      <c r="J77" t="n">
-        <v>-75.497944</v>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -13046,12 +12471,6 @@
           <t>JAUJA</t>
         </is>
       </c>
-      <c r="I78" t="n">
-        <v>-11.7676</v>
-      </c>
-      <c r="J78" t="n">
-        <v>-75.497944</v>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -13094,12 +12513,6 @@
           <t>JAUJA</t>
         </is>
       </c>
-      <c r="I79" t="n">
-        <v>-11.7676</v>
-      </c>
-      <c r="J79" t="n">
-        <v>-75.497944</v>
-      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -13142,12 +12555,6 @@
           <t>JUNIN</t>
         </is>
       </c>
-      <c r="I80" t="n">
-        <v>-11.161542</v>
-      </c>
-      <c r="J80" t="n">
-        <v>-75.99918599999999</v>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -13190,12 +12597,6 @@
           <t>JUNIN</t>
         </is>
       </c>
-      <c r="I81" t="n">
-        <v>-11.161542</v>
-      </c>
-      <c r="J81" t="n">
-        <v>-75.99918599999999</v>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -13238,12 +12639,6 @@
           <t>JUNIN</t>
         </is>
       </c>
-      <c r="I82" t="n">
-        <v>-11.161542</v>
-      </c>
-      <c r="J82" t="n">
-        <v>-75.99918599999999</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -13286,12 +12681,6 @@
           <t>JUNIN</t>
         </is>
       </c>
-      <c r="I83" t="n">
-        <v>-11.161542</v>
-      </c>
-      <c r="J83" t="n">
-        <v>-75.99918599999999</v>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -13334,12 +12723,6 @@
           <t>TARMA</t>
         </is>
       </c>
-      <c r="I84" t="n">
-        <v>-11.419558</v>
-      </c>
-      <c r="J84" t="n">
-        <v>-75.689481</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -13382,12 +12765,6 @@
           <t>TARMA</t>
         </is>
       </c>
-      <c r="I85" t="n">
-        <v>-11.418686</v>
-      </c>
-      <c r="J85" t="n">
-        <v>-75.698892</v>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -13430,12 +12807,6 @@
           <t>TARMA</t>
         </is>
       </c>
-      <c r="I86" t="n">
-        <v>-11.420861</v>
-      </c>
-      <c r="J86" t="n">
-        <v>-75.687747</v>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -13478,12 +12849,6 @@
           <t>TARMA</t>
         </is>
       </c>
-      <c r="I87" t="n">
-        <v>-11.420861</v>
-      </c>
-      <c r="J87" t="n">
-        <v>-75.687747</v>
-      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -13526,12 +12891,6 @@
           <t>TARMA</t>
         </is>
       </c>
-      <c r="I88" t="n">
-        <v>-11.420861</v>
-      </c>
-      <c r="J88" t="n">
-        <v>-75.687747</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -13574,12 +12933,6 @@
           <t>TARMA</t>
         </is>
       </c>
-      <c r="I89" t="n">
-        <v>-11.420861</v>
-      </c>
-      <c r="J89" t="n">
-        <v>-75.687747</v>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -13622,12 +12975,6 @@
           <t>TARMA</t>
         </is>
       </c>
-      <c r="I90" t="n">
-        <v>-11.420861</v>
-      </c>
-      <c r="J90" t="n">
-        <v>-75.687747</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -13670,12 +13017,6 @@
           <t>TARMA</t>
         </is>
       </c>
-      <c r="I91" t="n">
-        <v>-11.428728</v>
-      </c>
-      <c r="J91" t="n">
-        <v>-75.69157199999999</v>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -13718,12 +13059,6 @@
           <t>TARMA</t>
         </is>
       </c>
-      <c r="I92" t="n">
-        <v>-11.418686</v>
-      </c>
-      <c r="J92" t="n">
-        <v>-75.698892</v>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -13766,12 +13101,6 @@
           <t>ACOBAMBA</t>
         </is>
       </c>
-      <c r="I93" t="n">
-        <v>-11.354231</v>
-      </c>
-      <c r="J93" t="n">
-        <v>-75.65878600000001</v>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -13814,12 +13143,6 @@
           <t>LA OROYA</t>
         </is>
       </c>
-      <c r="I94" t="n">
-        <v>-11.521967</v>
-      </c>
-      <c r="J94" t="n">
-        <v>-75.908011</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -13862,12 +13185,6 @@
           <t>LA OROYA</t>
         </is>
       </c>
-      <c r="I95" t="n">
-        <v>-11.521967</v>
-      </c>
-      <c r="J95" t="n">
-        <v>-75.908011</v>
-      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -13910,12 +13227,6 @@
           <t>LA OROYA</t>
         </is>
       </c>
-      <c r="I96" t="n">
-        <v>-11.521967</v>
-      </c>
-      <c r="J96" t="n">
-        <v>-75.908011</v>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -13958,12 +13269,6 @@
           <t>LA OROYA</t>
         </is>
       </c>
-      <c r="I97" t="n">
-        <v>-11.521967</v>
-      </c>
-      <c r="J97" t="n">
-        <v>-75.908011</v>
-      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -14006,12 +13311,6 @@
           <t>PAMPAS</t>
         </is>
       </c>
-      <c r="I98" t="n">
-        <v>-12.400567</v>
-      </c>
-      <c r="J98" t="n">
-        <v>-74.874197</v>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -14054,12 +13353,6 @@
           <t>PAMPAS</t>
         </is>
       </c>
-      <c r="I99" t="n">
-        <v>-12.400567</v>
-      </c>
-      <c r="J99" t="n">
-        <v>-74.874197</v>
-      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -14102,12 +13395,6 @@
           <t>PAMPAS</t>
         </is>
       </c>
-      <c r="I100" t="n">
-        <v>-12.400567</v>
-      </c>
-      <c r="J100" t="n">
-        <v>-74.874197</v>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -14150,12 +13437,6 @@
           <t>PAMPAS</t>
         </is>
       </c>
-      <c r="I101" t="n">
-        <v>-12.400567</v>
-      </c>
-      <c r="J101" t="n">
-        <v>-74.874197</v>
-      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -14197,12 +13478,6 @@
         <is>
           <t>SURCUBAMBA</t>
         </is>
-      </c>
-      <c r="I102" t="n">
-        <v>-12.399214</v>
-      </c>
-      <c r="J102" t="n">
-        <v>-74.868161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Proyección poblacional sin Churcampa
</commit_message>
<xml_diff>
--- a/dashboard.xlsx
+++ b/dashboard.xlsx
@@ -196,7 +196,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="t_Poblacion" displayName="t_Poblacion" ref="A1:E55" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="t_Poblacion" displayName="t_Poblacion" ref="A1:E49" headerRowCount="1">
   <autoFilter ref="A1:E49"/>
   <tableColumns count="5">
     <tableColumn id="1" name="DEPARTAMENTO"/>
@@ -12276,7 +12276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -13318,132 +13318,6 @@
       </c>
       <c r="E49" t="n">
         <v>42704</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>HUANCAVELICA</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Churcampa (3 distritos)</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D50" t="n">
-        <v>4866</v>
-      </c>
-      <c r="E50" t="n">
-        <v>4963</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>HUANCAVELICA</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Churcampa (3 distritos)</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>2027</v>
-      </c>
-      <c r="D51" t="n">
-        <v>4924</v>
-      </c>
-      <c r="E51" t="n">
-        <v>5022</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>HUANCAVELICA</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Churcampa (3 distritos)</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
-        <v>2028</v>
-      </c>
-      <c r="D52" t="n">
-        <v>4983</v>
-      </c>
-      <c r="E52" t="n">
-        <v>5082</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>HUANCAVELICA</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Churcampa (3 distritos)</t>
-        </is>
-      </c>
-      <c r="C53" t="n">
-        <v>2029</v>
-      </c>
-      <c r="D53" t="n">
-        <v>5043</v>
-      </c>
-      <c r="E53" t="n">
-        <v>5142</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>HUANCAVELICA</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Churcampa (3 distritos)</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>2030</v>
-      </c>
-      <c r="D54" t="n">
-        <v>5103</v>
-      </c>
-      <c r="E54" t="n">
-        <v>5203</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>HUANCAVELICA</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Churcampa (3 distritos)</t>
-        </is>
-      </c>
-      <c r="C55" t="n">
-        <v>2031</v>
-      </c>
-      <c r="D55" t="n">
-        <v>5163</v>
-      </c>
-      <c r="E55" t="n">
-        <v>5266</v>
       </c>
     </row>
   </sheetData>

</xml_diff>